<commit_message>
Opérations : partenariats stratégiques, fiches process PR-01 à PR-10 et rétroplanning type (28/10/2026)
- Partenariats : cartographie des pistes par catégorie (Rungis, OneStaff,
  StaffMe, ProKitchens et alternatives, transport frigorifique, Options),
  grille de sélection et plan d'approche en quatre étapes. Aucun contact
  pris.
- Fiches process : objectif, responsable, étapes, livrable et contrôle
  pour chacun des dix process, avec les renforts C2 et C3.
- Rétroplanning type (Excel) : 24 jalons datés à partir de la date J et
  de la criticité, alertes de retard.
- Démarrage recommandé harmonisé à 8, 10 et 12 semaines (C1, C2, C3)
  dans la note de typologie et le calculateur de staffing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jw3cAQP549F4ThK9WHT6VD
</commit_message>
<xml_diff>
--- a/6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx
+++ b/6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="192">
   <si>
     <t xml:space="preserve">Calculateur de staffing par événement — Fou d'un soir</t>
   </si>
@@ -235,7 +235,7 @@
     <t xml:space="preserve">Dans le périmètre ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Délai minimum de préparation (semaines)</t>
+    <t xml:space="preserve">Démarrage recommandé (semaines avant J)</t>
   </si>
   <si>
     <t xml:space="preserve">Assiettes à laver (couverts × services)</t>
@@ -412,9 +412,6 @@
     <t xml:space="preserve">Niveau</t>
   </si>
   <si>
-    <t xml:space="preserve">Délai minimum (semaines)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Critères (il suffit d'en remplir un)</t>
   </si>
   <si>
@@ -424,19 +421,19 @@
     <t xml:space="preserve">Standard</t>
   </si>
   <si>
-    <t xml:space="preserve">Soirée récurrente vendue à la place ; chef et lieu déjà connus ; pas de presse. Délai : plan des pilotes du Produit (ventes à S-6).</t>
+    <t xml:space="preserve">Soirée récurrente vendue à la place ; chef et lieu déjà connus ; pas de presse. Démarrage : contrats signés avant l'ouverture des ventes, à S-6 (plan des pilotes du Produit), soit S-8.</t>
   </si>
   <si>
     <t xml:space="preserve">Premium</t>
   </si>
   <si>
-    <t xml:space="preserve">Client-payeur unique sous contrat ; chef étoilé ou étranger ; première collaboration avec un lieu ou un chef ; produits importés. Délai : plan des pilotes (lieux et chefs à S-10, contrats à S-8).</t>
+    <t xml:space="preserve">Client-payeur unique sous contrat ; chef étoilé ou étranger ; première collaboration avec un lieu ou un chef ; produits importés. Démarrage : lieux et chefs à S-10 (plan des pilotes du Produit).</t>
   </si>
   <si>
     <t xml:space="preserve">Signature</t>
   </si>
   <si>
-    <t xml:space="preserve">Presse, influenceurs ou célébrités ; maison de luxe sous contrat cadre ; lieu atypique ; soirée de lancement. Délai : 10 semaines et plus.</t>
+    <t xml:space="preserve">Presse, influenceurs ou célébrités ; maison de luxe sous contrat cadre ; lieu atypique ; soirée de lancement. Démarrage : S-12 (P).</t>
   </si>
   <si>
     <t xml:space="preserve">Rôles : heures et coûts (à renseigner à réception des devis)</t>
@@ -840,8 +837,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -861,23 +862,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -885,7 +886,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -893,7 +894,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -901,11 +902,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -921,7 +922,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -941,7 +942,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -953,7 +954,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1212,98 +1213,98 @@
   <dimension ref="A1:A20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="120"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1326,1640 +1327,1640 @@
   <dimension ref="A1:I56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="1" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="I6" s="10"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="I7" s="10"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="10" t="n">
+      <c r="C11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
+      <c r="G11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="I12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I13" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="I13" s="11"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12" t="str">
+      <c r="B16" s="12"/>
+      <c r="C16" s="13" t="str">
         <f aca="false">IF(C7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=C7,0),0)))</f>
         <v>T3</v>
       </c>
-      <c r="D16" s="12" t="str">
+      <c r="D16" s="13" t="str">
         <f aca="false">IF(D7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=D7,0),0)))</f>
         <v>T3</v>
       </c>
-      <c r="E16" s="12" t="str">
+      <c r="E16" s="13" t="str">
         <f aca="false">IF(E7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=E7,0),0)))</f>
         <v>T3</v>
       </c>
-      <c r="F16" s="12" t="str">
+      <c r="F16" s="13" t="str">
         <f aca="false">IF(F7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=F7,0),0)))</f>
         <v>T3</v>
       </c>
-      <c r="G16" s="12" t="str">
+      <c r="G16" s="13" t="str">
         <f aca="false">IF(G7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=G7,0),0)))</f>
         <v>T1</v>
       </c>
-      <c r="H16" s="12" t="str">
+      <c r="H16" s="13" t="str">
         <f aca="false">IF(H7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=H7,0),0)))</f>
         <v>T2</v>
       </c>
-      <c r="I16" s="12" t="str">
+      <c r="I16" s="13" t="str">
         <f aca="false">IF(I7="","",INDEX(Paramètres!$A$19:$A$23,MATCH(TRUE(),INDEX(Paramètres!$B$19:$B$23&gt;=I7,0),0)))</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12" t="str">
+      <c r="B17" s="12"/>
+      <c r="C17" s="13" t="str">
         <f aca="false">IF(OR(C7="",C10=""),"",C16&amp;" / "&amp;C10)</f>
         <v>T3 / C2</v>
       </c>
-      <c r="D17" s="12" t="str">
+      <c r="D17" s="13" t="str">
         <f aca="false">IF(OR(D7="",D10=""),"",D16&amp;" / "&amp;D10)</f>
         <v>T3 / C2</v>
       </c>
-      <c r="E17" s="12" t="str">
+      <c r="E17" s="13" t="str">
         <f aca="false">IF(OR(E7="",E10=""),"",E16&amp;" / "&amp;E10)</f>
         <v>T3 / C2</v>
       </c>
-      <c r="F17" s="12" t="str">
+      <c r="F17" s="13" t="str">
         <f aca="false">IF(OR(F7="",F10=""),"",F16&amp;" / "&amp;F10)</f>
         <v>T3 / C3</v>
       </c>
-      <c r="G17" s="12" t="str">
+      <c r="G17" s="13" t="str">
         <f aca="false">IF(OR(G7="",G10=""),"",G16&amp;" / "&amp;G10)</f>
         <v>T1 / C2</v>
       </c>
-      <c r="H17" s="12" t="str">
+      <c r="H17" s="13" t="str">
         <f aca="false">IF(OR(H7="",H10=""),"",H16&amp;" / "&amp;H10)</f>
         <v>T2 / C2</v>
       </c>
-      <c r="I17" s="12" t="str">
+      <c r="I17" s="13" t="str">
         <f aca="false">IF(OR(I7="",I10=""),"",I16&amp;" / "&amp;I10)</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="12" t="str">
+      <c r="B18" s="12"/>
+      <c r="C18" s="13" t="str">
         <f aca="false">IF(C16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(C16,Paramètres!$A$19:$A$23,0)))</f>
         <v>Oui : cœur de l'offre</v>
       </c>
-      <c r="D18" s="12" t="str">
+      <c r="D18" s="13" t="str">
         <f aca="false">IF(D16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(D16,Paramètres!$A$19:$A$23,0)))</f>
         <v>Oui : cœur de l'offre</v>
       </c>
-      <c r="E18" s="12" t="str">
+      <c r="E18" s="13" t="str">
         <f aca="false">IF(E16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(E16,Paramètres!$A$19:$A$23,0)))</f>
         <v>Oui : cœur de l'offre</v>
       </c>
-      <c r="F18" s="12" t="str">
+      <c r="F18" s="13" t="str">
         <f aca="false">IF(F16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(F16,Paramètres!$A$19:$A$23,0)))</f>
         <v>Oui : cœur de l'offre</v>
       </c>
-      <c r="G18" s="12" t="str">
+      <c r="G18" s="13" t="str">
         <f aca="false">IF(G16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(G16,Paramètres!$A$19:$A$23,0)))</f>
         <v>Oui</v>
       </c>
-      <c r="H18" s="12" t="str">
+      <c r="H18" s="13" t="str">
         <f aca="false">IF(H16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(H16,Paramètres!$A$19:$A$23,0)))</f>
         <v>Oui</v>
       </c>
-      <c r="I18" s="12" t="str">
+      <c r="I18" s="13" t="str">
         <f aca="false">IF(I16="","",INDEX(Paramètres!$D$19:$D$23,MATCH(I16,Paramètres!$A$19:$A$23,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12" t="n">
+      <c r="B19" s="12"/>
+      <c r="C19" s="13" t="n">
         <f aca="false">IF(C10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(C10,Paramètres!$A$28:$A$30,0)))</f>
-        <v>8</v>
-      </c>
-      <c r="D19" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="13" t="n">
         <f aca="false">IF(D10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(D10,Paramètres!$A$28:$A$30,0)))</f>
-        <v>8</v>
-      </c>
-      <c r="E19" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" s="13" t="n">
         <f aca="false">IF(E10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(E10,Paramètres!$A$28:$A$30,0)))</f>
-        <v>8</v>
-      </c>
-      <c r="F19" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" s="13" t="n">
         <f aca="false">IF(F10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(F10,Paramètres!$A$28:$A$30,0)))</f>
+        <v>12</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <f aca="false">IF(G10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(G10,Paramètres!$A$28:$A$30,0)))</f>
         <v>10</v>
       </c>
-      <c r="G19" s="12" t="n">
-        <f aca="false">IF(G10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(G10,Paramètres!$A$28:$A$30,0)))</f>
-        <v>8</v>
-      </c>
-      <c r="H19" s="12" t="n">
+      <c r="H19" s="13" t="n">
         <f aca="false">IF(H10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(H10,Paramètres!$A$28:$A$30,0)))</f>
-        <v>8</v>
-      </c>
-      <c r="I19" s="12" t="str">
+        <v>10</v>
+      </c>
+      <c r="I19" s="13" t="str">
         <f aca="false">IF(I10="","",INDEX(Paramètres!$B$28:$B$30,MATCH(I10,Paramètres!$A$28:$A$30,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <f aca="false">IF(OR(C7="",C8=""),"",C7*C8)</f>
         <v>144</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <f aca="false">IF(OR(D7="",D8=""),"",D7*D8)</f>
         <v>180</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="13" t="n">
         <f aca="false">IF(OR(E7="",E8=""),"",E7*E8)</f>
         <v>168</v>
       </c>
-      <c r="F20" s="12" t="str">
+      <c r="F20" s="13" t="str">
         <f aca="false">IF(OR(F7="",F8=""),"",F7*F8)</f>
         <v/>
       </c>
-      <c r="G20" s="12" t="str">
+      <c r="G20" s="13" t="str">
         <f aca="false">IF(OR(G7="",G8=""),"",G7*G8)</f>
         <v/>
       </c>
-      <c r="H20" s="12" t="str">
+      <c r="H20" s="13" t="str">
         <f aca="false">IF(OR(H7="",H8=""),"",H7*H8)</f>
         <v/>
       </c>
-      <c r="I20" s="12" t="str">
+      <c r="I20" s="13" t="str">
         <f aca="false">IF(OR(I7="",I8=""),"",I7*I8)</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <f aca="false">IF(C7="","",C7*(N(C9)+1))</f>
         <v>120</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="13" t="n">
         <f aca="false">IF(D7="","",D7*(N(D9)+1))</f>
         <v>20</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="13" t="n">
         <f aca="false">IF(E7="","",E7*(N(E9)+1))</f>
         <v>24</v>
       </c>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="13" t="n">
         <f aca="false">IF(F7="","",F7*(N(F9)+1))</f>
         <v>30</v>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="G21" s="13" t="n">
         <f aca="false">IF(G7="","",G7*(N(G9)+1))</f>
         <v>2</v>
       </c>
-      <c r="H21" s="12" t="n">
+      <c r="H21" s="13" t="n">
         <f aca="false">IF(H7="","",H7*(N(H9)+1))</f>
         <v>10</v>
       </c>
-      <c r="I21" s="12" t="str">
+      <c r="I21" s="13" t="str">
         <f aca="false">IF(I7="","",I7*(N(I9)+1))</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="str">
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="str">
         <f aca="false">Paramètres!A34</f>
         <v>Chef invité</v>
       </c>
-      <c r="B24" s="14" t="str">
+      <c r="B24" s="15" t="str">
         <f aca="false">Paramètres!E34</f>
         <v>1 par événement. Son cachet n'est pas horaire : le saisir à part avec la Finance (donnée n° 2).</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C24" s="13" t="n">
         <f aca="false">IF(C$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="D24" s="13" t="n">
         <f aca="false">IF(D$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E24" s="13" t="n">
         <f aca="false">IF(E$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="F24" s="12" t="n">
+      <c r="F24" s="13" t="n">
         <f aca="false">IF(F$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="G24" s="12" t="n">
+      <c r="G24" s="13" t="n">
         <f aca="false">IF(G$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="H24" s="12" t="n">
+      <c r="H24" s="13" t="n">
         <f aca="false">IF(H$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="I24" s="12" t="str">
+      <c r="I24" s="13" t="str">
         <f aca="false">IF(I$7="","",1)</f>
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="str">
+    <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="str">
         <f aca="false">Paramètres!A35</f>
         <v>Brigade (second, commis)</v>
       </c>
-      <c r="B25" s="14" t="str">
+      <c r="B25" s="15" t="str">
         <f aca="false">Paramètres!E35</f>
         <v>Couverts ÷ couverts par membre de brigade, arrondi au supérieur.</v>
       </c>
-      <c r="C25" s="12" t="n">
+      <c r="C25" s="13" t="n">
         <f aca="false">IF(C$7="","",ROUNDUP(C$7/Paramètres!$B$6,0))</f>
         <v>3</v>
       </c>
-      <c r="D25" s="12" t="n">
+      <c r="D25" s="13" t="n">
         <f aca="false">IF(D$7="","",ROUNDUP(D$7/Paramètres!$B$6,0))</f>
         <v>2</v>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="13" t="n">
         <f aca="false">IF(E$7="","",ROUNDUP(E$7/Paramètres!$B$6,0))</f>
         <v>3</v>
       </c>
-      <c r="F25" s="12" t="n">
+      <c r="F25" s="13" t="n">
         <f aca="false">IF(F$7="","",ROUNDUP(F$7/Paramètres!$B$6,0))</f>
         <v>3</v>
       </c>
-      <c r="G25" s="12" t="n">
+      <c r="G25" s="13" t="n">
         <f aca="false">IF(G$7="","",ROUNDUP(G$7/Paramètres!$B$6,0))</f>
         <v>1</v>
       </c>
-      <c r="H25" s="12" t="n">
+      <c r="H25" s="13" t="n">
         <f aca="false">IF(H$7="","",ROUNDUP(H$7/Paramètres!$B$6,0))</f>
         <v>1</v>
       </c>
-      <c r="I25" s="12" t="str">
+      <c r="I25" s="13" t="str">
         <f aca="false">IF(I$7="","",ROUNDUP(I$7/Paramètres!$B$6,0))</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="str">
+    <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="str">
         <f aca="false">Paramètres!A36</f>
         <v>Maître d'hôtel</v>
       </c>
-      <c r="B26" s="14" t="str">
+      <c r="B26" s="15" t="str">
         <f aca="false">Paramètres!E36</f>
         <v>1 à partir du seuil, 2 au-delà du second seuil.</v>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="C26" s="13" t="n">
         <f aca="false">IF(C$7="","",(C$7&gt;=Paramètres!$B$7)*1+(C$7&gt;=Paramètres!$B$8)*1)</f>
         <v>1</v>
       </c>
-      <c r="D26" s="12" t="n">
+      <c r="D26" s="13" t="n">
         <f aca="false">IF(D$7="","",(D$7&gt;=Paramètres!$B$7)*1+(D$7&gt;=Paramètres!$B$8)*1)</f>
         <v>1</v>
       </c>
-      <c r="E26" s="12" t="n">
+      <c r="E26" s="13" t="n">
         <f aca="false">IF(E$7="","",(E$7&gt;=Paramètres!$B$7)*1+(E$7&gt;=Paramètres!$B$8)*1)</f>
         <v>1</v>
       </c>
-      <c r="F26" s="12" t="n">
+      <c r="F26" s="13" t="n">
         <f aca="false">IF(F$7="","",(F$7&gt;=Paramètres!$B$7)*1+(F$7&gt;=Paramètres!$B$8)*1)</f>
         <v>1</v>
       </c>
-      <c r="G26" s="12" t="n">
+      <c r="G26" s="13" t="n">
         <f aca="false">IF(G$7="","",(G$7&gt;=Paramètres!$B$7)*1+(G$7&gt;=Paramètres!$B$8)*1)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="12" t="n">
+      <c r="H26" s="13" t="n">
         <f aca="false">IF(H$7="","",(H$7&gt;=Paramètres!$B$7)*1+(H$7&gt;=Paramètres!$B$8)*1)</f>
         <v>1</v>
       </c>
-      <c r="I26" s="12" t="str">
+      <c r="I26" s="13" t="str">
         <f aca="false">IF(I$7="","",(I$7&gt;=Paramètres!$B$7)*1+(I$7&gt;=Paramètres!$B$8)*1)</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="str">
+    <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="str">
         <f aca="false">Paramètres!A37</f>
         <v>Serveurs (base)</v>
       </c>
-      <c r="B27" s="14" t="str">
+      <c r="B27" s="15" t="str">
         <f aca="false">Paramètres!E37</f>
         <v>Couverts ÷ couverts par serveur, arrondi au supérieur.</v>
       </c>
-      <c r="C27" s="12" t="n">
+      <c r="C27" s="13" t="n">
         <f aca="false">IF(C$7="","",ROUNDUP(C$7/Paramètres!$B$5,0))</f>
         <v>4</v>
       </c>
-      <c r="D27" s="12" t="n">
+      <c r="D27" s="13" t="n">
         <f aca="false">IF(D$7="","",ROUNDUP(D$7/Paramètres!$B$5,0))</f>
         <v>3</v>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="E27" s="13" t="n">
         <f aca="false">IF(E$7="","",ROUNDUP(E$7/Paramètres!$B$5,0))</f>
         <v>4</v>
       </c>
-      <c r="F27" s="12" t="n">
+      <c r="F27" s="13" t="n">
         <f aca="false">IF(F$7="","",ROUNDUP(F$7/Paramètres!$B$5,0))</f>
         <v>5</v>
       </c>
-      <c r="G27" s="12" t="n">
+      <c r="G27" s="13" t="n">
         <f aca="false">IF(G$7="","",ROUNDUP(G$7/Paramètres!$B$5,0))</f>
         <v>1</v>
       </c>
-      <c r="H27" s="12" t="n">
+      <c r="H27" s="13" t="n">
         <f aca="false">IF(H$7="","",ROUNDUP(H$7/Paramètres!$B$5,0))</f>
         <v>2</v>
       </c>
-      <c r="I27" s="12" t="str">
+      <c r="I27" s="13" t="str">
         <f aca="false">IF(I$7="","",ROUNDUP(I$7/Paramètres!$B$5,0))</f>
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="str">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="str">
         <f aca="false">Paramètres!A38</f>
         <v>Serveur de réserve</v>
       </c>
-      <c r="B28" s="14" t="str">
+      <c r="B28" s="15" t="str">
         <f aca="false">Paramètres!E38</f>
         <v>1 en C2 et en C3.</v>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(OR(C$10="C2",C$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="D28" s="12" t="n">
+      <c r="D28" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(OR(D$10="C2",D$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="E28" s="12" t="n">
+      <c r="E28" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(OR(E$10="C2",E$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="F28" s="12" t="n">
+      <c r="F28" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(OR(F$10="C2",F$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="G28" s="12" t="n">
+      <c r="G28" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(OR(G$10="C2",G$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="H28" s="12" t="n">
+      <c r="H28" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(OR(H$10="C2",H$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="I28" s="12" t="str">
+      <c r="I28" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(OR(I$10="C2",I$10="C3"),1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="str">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="str">
         <f aca="false">Paramètres!A39</f>
         <v>Serveurs pour salons supplémentaires</v>
       </c>
-      <c r="B29" s="14" t="str">
+      <c r="B29" s="15" t="str">
         <f aca="false">Paramètres!E39</f>
         <v>En C3 : 1 par salon au-delà du premier.</v>
       </c>
-      <c r="C29" s="12" t="n">
+      <c r="C29" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(C$10="C3",MAX(N(C$11)-1,0),0))</f>
         <v>0</v>
       </c>
-      <c r="D29" s="12" t="n">
+      <c r="D29" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(D$10="C3",MAX(N(D$11)-1,0),0))</f>
         <v>0</v>
       </c>
-      <c r="E29" s="12" t="n">
+      <c r="E29" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(E$10="C3",MAX(N(E$11)-1,0),0))</f>
         <v>0</v>
       </c>
-      <c r="F29" s="12" t="n">
+      <c r="F29" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(F$10="C3",MAX(N(F$11)-1,0),0))</f>
         <v>2</v>
       </c>
-      <c r="G29" s="12" t="n">
+      <c r="G29" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(G$10="C3",MAX(N(G$11)-1,0),0))</f>
         <v>0</v>
       </c>
-      <c r="H29" s="12" t="n">
+      <c r="H29" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(H$10="C3",MAX(N(H$11)-1,0),0))</f>
         <v>0</v>
       </c>
-      <c r="I29" s="12" t="str">
+      <c r="I29" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(I$10="C3",MAX(N(I$11)-1,0),0))</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="str">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="str">
         <f aca="false">Paramètres!A40</f>
         <v>Sommelier invité</v>
       </c>
-      <c r="B30" s="14" t="str">
+      <c r="B30" s="15" t="str">
         <f aca="false">Paramètres!E40</f>
         <v>1 par événement.</v>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="13" t="n">
         <f aca="false">IF(C$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="D30" s="12" t="n">
+      <c r="D30" s="13" t="n">
         <f aca="false">IF(D$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="E30" s="12" t="n">
+      <c r="E30" s="13" t="n">
         <f aca="false">IF(E$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="F30" s="12" t="n">
+      <c r="F30" s="13" t="n">
         <f aca="false">IF(F$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="G30" s="12" t="n">
+      <c r="G30" s="13" t="n">
         <f aca="false">IF(G$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="H30" s="12" t="n">
+      <c r="H30" s="13" t="n">
         <f aca="false">IF(H$7="","",1)</f>
         <v>1</v>
       </c>
-      <c r="I30" s="12" t="str">
+      <c r="I30" s="13" t="str">
         <f aca="false">IF(I$7="","",1)</f>
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="str">
+    <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="14" t="str">
         <f aca="false">Paramètres!A41</f>
         <v>Aide sommelier</v>
       </c>
-      <c r="B31" s="14" t="str">
+      <c r="B31" s="15" t="str">
         <f aca="false">Paramètres!E41</f>
         <v>1 à partir du seuil, 2 au-delà du second seuil.</v>
       </c>
-      <c r="C31" s="12" t="n">
+      <c r="C31" s="13" t="n">
         <f aca="false">IF(C$7="","",(C$7&gt;=Paramètres!$B$9)*1+(C$7&gt;=Paramètres!$B$10)*1)</f>
         <v>1</v>
       </c>
-      <c r="D31" s="12" t="n">
+      <c r="D31" s="13" t="n">
         <f aca="false">IF(D$7="","",(D$7&gt;=Paramètres!$B$9)*1+(D$7&gt;=Paramètres!$B$10)*1)</f>
         <v>1</v>
       </c>
-      <c r="E31" s="12" t="n">
+      <c r="E31" s="13" t="n">
         <f aca="false">IF(E$7="","",(E$7&gt;=Paramètres!$B$9)*1+(E$7&gt;=Paramètres!$B$10)*1)</f>
         <v>1</v>
       </c>
-      <c r="F31" s="12" t="n">
+      <c r="F31" s="13" t="n">
         <f aca="false">IF(F$7="","",(F$7&gt;=Paramètres!$B$9)*1+(F$7&gt;=Paramètres!$B$10)*1)</f>
         <v>1</v>
       </c>
-      <c r="G31" s="12" t="n">
+      <c r="G31" s="13" t="n">
         <f aca="false">IF(G$7="","",(G$7&gt;=Paramètres!$B$9)*1+(G$7&gt;=Paramètres!$B$10)*1)</f>
         <v>0</v>
       </c>
-      <c r="H31" s="12" t="n">
+      <c r="H31" s="13" t="n">
         <f aca="false">IF(H$7="","",(H$7&gt;=Paramètres!$B$9)*1+(H$7&gt;=Paramètres!$B$10)*1)</f>
         <v>0</v>
       </c>
-      <c r="I31" s="12" t="str">
+      <c r="I31" s="13" t="str">
         <f aca="false">IF(I$7="","",(I$7&gt;=Paramètres!$B$9)*1+(I$7&gt;=Paramètres!$B$10)*1)</f>
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="str">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="str">
         <f aca="false">Paramètres!A42</f>
         <v>Plongeurs</v>
       </c>
-      <c r="B32" s="14" t="str">
+      <c r="B32" s="15" t="str">
         <f aca="false">Paramètres!E42</f>
         <v>1, puis 2 et 3 selon les seuils.</v>
       </c>
-      <c r="C32" s="12" t="n">
+      <c r="C32" s="13" t="n">
         <f aca="false">IF(C$7="","",1+(C$7&gt;=Paramètres!$B$11)*1+(C$7&gt;=Paramètres!$B$12)*1)</f>
         <v>2</v>
       </c>
-      <c r="D32" s="12" t="n">
+      <c r="D32" s="13" t="n">
         <f aca="false">IF(D$7="","",1+(D$7&gt;=Paramètres!$B$11)*1+(D$7&gt;=Paramètres!$B$12)*1)</f>
         <v>2</v>
       </c>
-      <c r="E32" s="12" t="n">
+      <c r="E32" s="13" t="n">
         <f aca="false">IF(E$7="","",1+(E$7&gt;=Paramètres!$B$11)*1+(E$7&gt;=Paramètres!$B$12)*1)</f>
         <v>2</v>
       </c>
-      <c r="F32" s="12" t="n">
+      <c r="F32" s="13" t="n">
         <f aca="false">IF(F$7="","",1+(F$7&gt;=Paramètres!$B$11)*1+(F$7&gt;=Paramètres!$B$12)*1)</f>
         <v>2</v>
       </c>
-      <c r="G32" s="12" t="n">
+      <c r="G32" s="13" t="n">
         <f aca="false">IF(G$7="","",1+(G$7&gt;=Paramètres!$B$11)*1+(G$7&gt;=Paramètres!$B$12)*1)</f>
         <v>1</v>
       </c>
-      <c r="H32" s="12" t="n">
+      <c r="H32" s="13" t="n">
         <f aca="false">IF(H$7="","",1+(H$7&gt;=Paramètres!$B$11)*1+(H$7&gt;=Paramètres!$B$12)*1)</f>
         <v>1</v>
       </c>
-      <c r="I32" s="12" t="str">
+      <c r="I32" s="13" t="str">
         <f aca="false">IF(I$7="","",1+(I$7&gt;=Paramètres!$B$11)*1+(I$7&gt;=Paramètres!$B$12)*1)</f>
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="str">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="str">
         <f aca="false">Paramètres!A43</f>
         <v>Responsable de production (nous)</v>
       </c>
-      <c r="B33" s="14" t="str">
+      <c r="B33" s="15" t="str">
         <f aca="false">Paramètres!E43</f>
         <v>1, puis 2 à partir du seuil.</v>
       </c>
-      <c r="C33" s="12" t="n">
+      <c r="C33" s="13" t="n">
         <f aca="false">IF(C$7="","",1+(C$7&gt;=Paramètres!$B$13)*1)</f>
         <v>1</v>
       </c>
-      <c r="D33" s="12" t="n">
+      <c r="D33" s="13" t="n">
         <f aca="false">IF(D$7="","",1+(D$7&gt;=Paramètres!$B$13)*1)</f>
         <v>1</v>
       </c>
-      <c r="E33" s="12" t="n">
+      <c r="E33" s="13" t="n">
         <f aca="false">IF(E$7="","",1+(E$7&gt;=Paramètres!$B$13)*1)</f>
         <v>1</v>
       </c>
-      <c r="F33" s="12" t="n">
+      <c r="F33" s="13" t="n">
         <f aca="false">IF(F$7="","",1+(F$7&gt;=Paramètres!$B$13)*1)</f>
         <v>1</v>
       </c>
-      <c r="G33" s="12" t="n">
+      <c r="G33" s="13" t="n">
         <f aca="false">IF(G$7="","",1+(G$7&gt;=Paramètres!$B$13)*1)</f>
         <v>1</v>
       </c>
-      <c r="H33" s="12" t="n">
+      <c r="H33" s="13" t="n">
         <f aca="false">IF(H$7="","",1+(H$7&gt;=Paramètres!$B$13)*1)</f>
         <v>1</v>
       </c>
-      <c r="I33" s="12" t="str">
+      <c r="I33" s="13" t="str">
         <f aca="false">IF(I$7="","",1+(I$7&gt;=Paramètres!$B$13)*1)</f>
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="str">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="str">
         <f aca="false">Paramètres!A44</f>
         <v>Interlocuteur client (Ventes)</v>
       </c>
-      <c r="B34" s="14" t="str">
+      <c r="B34" s="15" t="str">
         <f aca="false">Paramètres!E44</f>
         <v>1 en C2 et en C3.</v>
       </c>
-      <c r="C34" s="12" t="n">
+      <c r="C34" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(OR(C$10="C2",C$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="D34" s="12" t="n">
+      <c r="D34" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(OR(D$10="C2",D$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="E34" s="12" t="n">
+      <c r="E34" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(OR(E$10="C2",E$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="F34" s="12" t="n">
+      <c r="F34" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(OR(F$10="C2",F$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="G34" s="12" t="n">
+      <c r="G34" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(OR(G$10="C2",G$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="H34" s="12" t="n">
+      <c r="H34" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(OR(H$10="C2",H$10="C3"),1,0))</f>
         <v>1</v>
       </c>
-      <c r="I34" s="12" t="str">
+      <c r="I34" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(OR(I$10="C2",I$10="C3"),1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="str">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="str">
         <f aca="false">Paramètres!A45</f>
         <v>Accueil et vestiaire</v>
       </c>
-      <c r="B35" s="14" t="str">
+      <c r="B35" s="15" t="str">
         <f aca="false">Paramètres!E45</f>
         <v>En C3 : 1, puis 2 à partir du seuil.</v>
       </c>
-      <c r="C35" s="12" t="n">
+      <c r="C35" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(C$10="C3",1+(C$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v>0</v>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D35" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(D$10="C3",1+(D$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v>0</v>
       </c>
-      <c r="E35" s="12" t="n">
+      <c r="E35" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(E$10="C3",1+(E$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v>0</v>
       </c>
-      <c r="F35" s="12" t="n">
+      <c r="F35" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(F$10="C3",1+(F$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v>1</v>
       </c>
-      <c r="G35" s="12" t="n">
+      <c r="G35" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(G$10="C3",1+(G$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v>0</v>
       </c>
-      <c r="H35" s="12" t="n">
+      <c r="H35" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(H$10="C3",1+(H$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v>0</v>
       </c>
-      <c r="I35" s="12" t="str">
+      <c r="I35" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(I$10="C3",1+(I$7&gt;=Paramètres!$B$14)*1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="str">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="str">
         <f aca="false">Paramètres!A46</f>
         <v>Relations presse et invités (Marketing)</v>
       </c>
-      <c r="B36" s="14" t="str">
+      <c r="B36" s="15" t="str">
         <f aca="false">Paramètres!E46</f>
         <v>1 en C3.</v>
       </c>
-      <c r="C36" s="12" t="n">
+      <c r="C36" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(C$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D36" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(D$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="E36" s="12" t="n">
+      <c r="E36" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(E$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="F36" s="12" t="n">
+      <c r="F36" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(F$10="C3",1,0))</f>
         <v>1</v>
       </c>
-      <c r="G36" s="12" t="n">
+      <c r="G36" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(G$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="H36" s="12" t="n">
+      <c r="H36" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(H$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="I36" s="12" t="str">
+      <c r="I36" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(I$10="C3",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="str">
+    <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="str">
         <f aca="false">Paramètres!A47</f>
         <v>Photographe</v>
       </c>
-      <c r="B37" s="14" t="str">
+      <c r="B37" s="15" t="str">
         <f aca="false">Paramètres!E47</f>
         <v>1 en C3 (prévu dans les trois options de lancement du Marketing).</v>
       </c>
-      <c r="C37" s="12" t="n">
+      <c r="C37" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(C$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="D37" s="12" t="n">
+      <c r="D37" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(D$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="E37" s="12" t="n">
+      <c r="E37" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(E$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="F37" s="12" t="n">
+      <c r="F37" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(F$10="C3",1,0))</f>
         <v>1</v>
       </c>
-      <c r="G37" s="12" t="n">
+      <c r="G37" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(G$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="H37" s="12" t="n">
+      <c r="H37" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(H$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="I37" s="12" t="str">
+      <c r="I37" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(I$10="C3",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="str">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="str">
         <f aca="false">Paramètres!A48</f>
         <v>Vidéaste</v>
       </c>
-      <c r="B38" s="14" t="str">
+      <c r="B38" s="15" t="str">
         <f aca="false">Paramètres!E48</f>
         <v>1 en C3 (idem).</v>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(C$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D38" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(D$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="E38" s="12" t="n">
+      <c r="E38" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(E$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="F38" s="12" t="n">
+      <c r="F38" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(F$10="C3",1,0))</f>
         <v>1</v>
       </c>
-      <c r="G38" s="12" t="n">
+      <c r="G38" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(G$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="H38" s="12" t="n">
+      <c r="H38" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(H$10="C3",1,0))</f>
         <v>0</v>
       </c>
-      <c r="I38" s="12" t="str">
+      <c r="I38" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(I$10="C3",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="str">
+    <row r="39" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="str">
         <f aca="false">Paramètres!A49</f>
         <v>Logistique d'accès</v>
       </c>
-      <c r="B39" s="14" t="str">
+      <c r="B39" s="15" t="str">
         <f aca="false">Paramètres!E49</f>
         <v>1 si le lieu exige une logistique d'accès particulière (ex. bateaux).</v>
       </c>
-      <c r="C39" s="12" t="n">
+      <c r="C39" s="13" t="n">
         <f aca="false">IF(C$7="","",IF(C$12="Oui",1,0))</f>
         <v>0</v>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D39" s="13" t="n">
         <f aca="false">IF(D$7="","",IF(D$12="Oui",1,0))</f>
         <v>0</v>
       </c>
-      <c r="E39" s="12" t="n">
+      <c r="E39" s="13" t="n">
         <f aca="false">IF(E$7="","",IF(E$12="Oui",1,0))</f>
         <v>0</v>
       </c>
-      <c r="F39" s="12" t="n">
+      <c r="F39" s="13" t="n">
         <f aca="false">IF(F$7="","",IF(F$12="Oui",1,0))</f>
         <v>0</v>
       </c>
-      <c r="G39" s="12" t="n">
+      <c r="G39" s="13" t="n">
         <f aca="false">IF(G$7="","",IF(G$12="Oui",1,0))</f>
         <v>0</v>
       </c>
-      <c r="H39" s="12" t="n">
+      <c r="H39" s="13" t="n">
         <f aca="false">IF(H$7="","",IF(H$12="Oui",1,0))</f>
         <v>0</v>
       </c>
-      <c r="I39" s="12" t="str">
+      <c r="I39" s="13" t="str">
         <f aca="false">IF(I$7="","",IF(I$12="Oui",1,0))</f>
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B40" s="16"/>
-      <c r="C40" s="17" t="n">
+      <c r="B40" s="17"/>
+      <c r="C40" s="18" t="n">
         <f aca="false">IF(C7="","",SUM(C24:C39))</f>
         <v>16</v>
       </c>
-      <c r="D40" s="17" t="n">
+      <c r="D40" s="18" t="n">
         <f aca="false">IF(D7="","",SUM(D24:D39))</f>
         <v>14</v>
       </c>
-      <c r="E40" s="17" t="n">
+      <c r="E40" s="18" t="n">
         <f aca="false">IF(E7="","",SUM(E24:E39))</f>
         <v>16</v>
       </c>
-      <c r="F40" s="17" t="n">
+      <c r="F40" s="18" t="n">
         <f aca="false">IF(F7="","",SUM(F24:F39))</f>
         <v>23</v>
       </c>
-      <c r="G40" s="17" t="n">
+      <c r="G40" s="18" t="n">
         <f aca="false">IF(G7="","",SUM(G24:G39))</f>
         <v>8</v>
       </c>
-      <c r="H40" s="17" t="n">
+      <c r="H40" s="18" t="n">
         <f aca="false">IF(H7="","",SUM(H24:H39))</f>
         <v>10</v>
       </c>
-      <c r="I40" s="17" t="str">
+      <c r="I40" s="18" t="str">
         <f aca="false">IF(I7="","",SUM(I24:I39))</f>
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="8" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="18" t="n">
+      <c r="B41" s="12"/>
+      <c r="C41" s="19" t="n">
         <f aca="false">IF(C7="","",IF(C13="Restaurant",SUMPRODUCT(C24:C39,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="D41" s="18" t="n">
+      <c r="D41" s="19" t="n">
         <f aca="false">IF(D7="","",IF(D13="Restaurant",SUMPRODUCT(D24:D39,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="E41" s="18" t="n">
+      <c r="E41" s="19" t="n">
         <f aca="false">IF(E7="","",IF(E13="Restaurant",SUMPRODUCT(E24:E39,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="F41" s="18" t="n">
+      <c r="F41" s="19" t="n">
         <f aca="false">IF(F7="","",IF(F13="Restaurant",SUMPRODUCT(F24:F39,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="G41" s="18" t="n">
+      <c r="G41" s="19" t="n">
         <f aca="false">IF(G7="","",IF(G13="Restaurant",SUMPRODUCT(G24:G39,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="H41" s="18" t="n">
+      <c r="H41" s="19" t="n">
         <f aca="false">IF(H7="","",IF(H13="Restaurant",SUMPRODUCT(H24:H39,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="I41" s="18" t="str">
+      <c r="I41" s="19" t="str">
         <f aca="false">IF(I7="","",IF(I13="Restaurant",SUMPRODUCT(I24:I39,Paramètres!$D$34:$D$49),0))</f>
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="16"/>
-      <c r="C42" s="17" t="n">
+      <c r="B42" s="17"/>
+      <c r="C42" s="18" t="n">
         <f aca="false">IF(C7="","",C40-C41)</f>
         <v>16</v>
       </c>
-      <c r="D42" s="17" t="n">
+      <c r="D42" s="18" t="n">
         <f aca="false">IF(D7="","",D40-D41)</f>
         <v>14</v>
       </c>
-      <c r="E42" s="17" t="n">
+      <c r="E42" s="18" t="n">
         <f aca="false">IF(E7="","",E40-E41)</f>
         <v>16</v>
       </c>
-      <c r="F42" s="17" t="n">
+      <c r="F42" s="18" t="n">
         <f aca="false">IF(F7="","",F40-F41)</f>
         <v>23</v>
       </c>
-      <c r="G42" s="17" t="n">
+      <c r="G42" s="18" t="n">
         <f aca="false">IF(G7="","",G40-G41)</f>
         <v>8</v>
       </c>
-      <c r="H42" s="17" t="n">
+      <c r="H42" s="18" t="n">
         <f aca="false">IF(H7="","",H40-H41)</f>
         <v>10</v>
       </c>
-      <c r="I42" s="17" t="str">
+      <c r="I42" s="18" t="str">
         <f aca="false">IF(I7="","",I40-I41)</f>
         <v/>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="8" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C43" s="19" t="n">
+      <c r="C43" s="20" t="n">
         <f aca="false">IF(C7="","",SUMPRODUCT(C24:C39,Paramètres!$B$34:$B$49)-IF(C13="Restaurant",SUMPRODUCT(C24:C39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="D43" s="19" t="n">
+      <c r="D43" s="20" t="n">
         <f aca="false">IF(D7="","",SUMPRODUCT(D24:D39,Paramètres!$B$34:$B$49)-IF(D13="Restaurant",SUMPRODUCT(D24:D39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="E43" s="19" t="n">
+      <c r="E43" s="20" t="n">
         <f aca="false">IF(E7="","",SUMPRODUCT(E24:E39,Paramètres!$B$34:$B$49)-IF(E13="Restaurant",SUMPRODUCT(E24:E39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="F43" s="19" t="n">
+      <c r="F43" s="20" t="n">
         <f aca="false">IF(F7="","",SUMPRODUCT(F24:F39,Paramètres!$B$34:$B$49)-IF(F13="Restaurant",SUMPRODUCT(F24:F39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="G43" s="19" t="n">
+      <c r="G43" s="20" t="n">
         <f aca="false">IF(G7="","",SUMPRODUCT(G24:G39,Paramètres!$B$34:$B$49)-IF(G13="Restaurant",SUMPRODUCT(G24:G39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="H43" s="19" t="n">
+      <c r="H43" s="20" t="n">
         <f aca="false">IF(H7="","",SUMPRODUCT(H24:H39,Paramètres!$B$34:$B$49)-IF(H13="Restaurant",SUMPRODUCT(H24:H39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="I43" s="19" t="str">
+      <c r="I43" s="20" t="str">
         <f aca="false">IF(I7="","",SUMPRODUCT(I24:I39,Paramètres!$B$34:$B$49)-IF(I13="Restaurant",SUMPRODUCT(I24:I39,Paramètres!$B$34:$B$49,Paramètres!$D$34:$D$49),0))</f>
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="B44" s="20" t="s">
+      <c r="B44" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="21" t="n">
+      <c r="C44" s="22" t="n">
         <f aca="false">IF(C7="","",SUMPRODUCT(C24:C39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(C13="Restaurant",SUMPRODUCT(C24:C39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="D44" s="21" t="n">
+      <c r="D44" s="22" t="n">
         <f aca="false">IF(D7="","",SUMPRODUCT(D24:D39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(D13="Restaurant",SUMPRODUCT(D24:D39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="E44" s="21" t="n">
+      <c r="E44" s="22" t="n">
         <f aca="false">IF(E7="","",SUMPRODUCT(E24:E39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(E13="Restaurant",SUMPRODUCT(E24:E39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="F44" s="21" t="n">
+      <c r="F44" s="22" t="n">
         <f aca="false">IF(F7="","",SUMPRODUCT(F24:F39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(F13="Restaurant",SUMPRODUCT(F24:F39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="G44" s="21" t="n">
+      <c r="G44" s="22" t="n">
         <f aca="false">IF(G7="","",SUMPRODUCT(G24:G39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(G13="Restaurant",SUMPRODUCT(G24:G39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="H44" s="21" t="n">
+      <c r="H44" s="22" t="n">
         <f aca="false">IF(H7="","",SUMPRODUCT(H24:H39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(H13="Restaurant",SUMPRODUCT(H24:H39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v>0</v>
       </c>
-      <c r="I44" s="21" t="str">
+      <c r="I44" s="22" t="str">
         <f aca="false">IF(I7="","",SUMPRODUCT(I24:I39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49)-IF(I13="Restaurant",SUMPRODUCT(I24:I39,Paramètres!$B$34:$B$49,Paramètres!$C$34:$C$49,Paramètres!$D$34:$D$49),0))</f>
         <v/>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
-    </row>
-    <row r="47" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="13" t="str">
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
+      <c r="I46" s="8"/>
+    </row>
+    <row r="47" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="str">
         <f aca="false">Paramètres!A55</f>
         <v>PR-01 Qualification du lieu</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="22" t="str">
+      <c r="B47" s="12"/>
+      <c r="C47" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ visite sur place</v>
       </c>
-      <c r="D47" s="22" t="str">
+      <c r="D47" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ visite sur place</v>
       </c>
-      <c r="E47" s="22" t="str">
+      <c r="E47" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ visite sur place</v>
       </c>
-      <c r="F47" s="22" t="str">
+      <c r="F47" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ visite technique et répétition sur place</v>
       </c>
-      <c r="G47" s="22" t="str">
+      <c r="G47" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ visite sur place</v>
       </c>
-      <c r="H47" s="22" t="str">
+      <c r="H47" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ visite sur place</v>
       </c>
-      <c r="I47" s="22" t="str">
+      <c r="I47" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$55:$D$55,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13" t="str">
+    <row r="48" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="str">
         <f aca="false">Paramètres!A56</f>
         <v>PR-02 Engagement du chef</v>
       </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="22" t="str">
+      <c r="B48" s="12"/>
+      <c r="C48" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ chef de secours désigné par écrit</v>
       </c>
-      <c r="D48" s="22" t="str">
+      <c r="D48" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ chef de secours désigné par écrit</v>
       </c>
-      <c r="E48" s="22" t="str">
+      <c r="E48" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ chef de secours désigné par écrit</v>
       </c>
-      <c r="F48" s="22" t="str">
+      <c r="F48" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + accord écrit sur la communication autour du chef</v>
       </c>
-      <c r="G48" s="22" t="str">
+      <c r="G48" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ chef de secours désigné par écrit</v>
       </c>
-      <c r="H48" s="22" t="str">
+      <c r="H48" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ chef de secours désigné par écrit</v>
       </c>
-      <c r="I48" s="22" t="str">
+      <c r="I48" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$56:$D$56,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13" t="str">
+    <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="str">
         <f aca="false">Paramètres!A57</f>
         <v>PR-03 Fiche technique de l'événement</v>
       </c>
-      <c r="B49" s="11"/>
-      <c r="C49" s="22" t="str">
+      <c r="B49" s="12"/>
+      <c r="C49" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ validée par le client</v>
       </c>
-      <c r="D49" s="22" t="str">
+      <c r="D49" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ validée par le client</v>
       </c>
-      <c r="E49" s="22" t="str">
+      <c r="E49" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ validée par le client</v>
       </c>
-      <c r="F49" s="22" t="str">
+      <c r="F49" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + liste des invités et confidentialité</v>
       </c>
-      <c r="G49" s="22" t="str">
+      <c r="G49" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ validée par le client</v>
       </c>
-      <c r="H49" s="22" t="str">
+      <c r="H49" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ validée par le client</v>
       </c>
-      <c r="I49" s="22" t="str">
+      <c r="I49" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$57:$D$57,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="13" t="str">
+    <row r="50" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="str">
         <f aca="false">Paramètres!A58</f>
         <v>PR-04 Staffing</v>
       </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="22" t="str">
+      <c r="B50" s="12"/>
+      <c r="C50" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + 1 personne de réserve</v>
       </c>
-      <c r="D50" s="22" t="str">
+      <c r="D50" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + 1 personne de réserve</v>
       </c>
-      <c r="E50" s="22" t="str">
+      <c r="E50" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + 1 personne de réserve</v>
       </c>
-      <c r="F50" s="22" t="str">
+      <c r="F50" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + accueil, presse, images</v>
       </c>
-      <c r="G50" s="22" t="str">
+      <c r="G50" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + 1 personne de réserve</v>
       </c>
-      <c r="H50" s="22" t="str">
+      <c r="H50" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + 1 personne de réserve</v>
       </c>
-      <c r="I50" s="22" t="str">
+      <c r="I50" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$58:$D$58,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="13" t="str">
+    <row r="51" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="str">
         <f aca="false">Paramètres!A59</f>
         <v>PR-05 Achats et approvisionnement</v>
       </c>
-      <c r="B51" s="11"/>
-      <c r="C51" s="22" t="str">
+      <c r="B51" s="12"/>
+      <c r="C51" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ fournisseur de secours identifié</v>
       </c>
-      <c r="D51" s="22" t="str">
+      <c r="D51" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ fournisseur de secours identifié</v>
       </c>
-      <c r="E51" s="22" t="str">
+      <c r="E51" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ fournisseur de secours identifié</v>
       </c>
-      <c r="F51" s="22" t="str">
+      <c r="F51" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + importations anticipées</v>
       </c>
-      <c r="G51" s="22" t="str">
+      <c r="G51" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ fournisseur de secours identifié</v>
       </c>
-      <c r="H51" s="22" t="str">
+      <c r="H51" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ fournisseur de secours identifié</v>
       </c>
-      <c r="I51" s="22" t="str">
+      <c r="I51" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$59:$D$59,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="13" t="str">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="str">
         <f aca="false">Paramètres!A60</f>
         <v>PR-06 Hygiène et allergènes</v>
       </c>
-      <c r="B52" s="11"/>
-      <c r="C52" s="22" t="str">
+      <c r="B52" s="12"/>
+      <c r="C52" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="D52" s="22" t="str">
+      <c r="D52" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="E52" s="22" t="str">
+      <c r="E52" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="F52" s="22" t="str">
+      <c r="F52" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="G52" s="22" t="str">
+      <c r="G52" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="H52" s="22" t="str">
+      <c r="H52" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="I52" s="22" t="str">
+      <c r="I52" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$60:$D$60,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="13" t="str">
+    <row r="53" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="str">
         <f aca="false">Paramètres!A61</f>
         <v>PR-07 Déroulé du jour J</v>
       </c>
-      <c r="B53" s="11"/>
-      <c r="C53" s="22" t="str">
+      <c r="B53" s="12"/>
+      <c r="C53" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ déroulé partagé avec le client</v>
       </c>
-      <c r="D53" s="22" t="str">
+      <c r="D53" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ déroulé partagé avec le client</v>
       </c>
-      <c r="E53" s="22" t="str">
+      <c r="E53" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ déroulé partagé avec le client</v>
       </c>
-      <c r="F53" s="22" t="str">
+      <c r="F53" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + dégustation du menu à l'avance et répétition</v>
       </c>
-      <c r="G53" s="22" t="str">
+      <c r="G53" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ déroulé partagé avec le client</v>
       </c>
-      <c r="H53" s="22" t="str">
+      <c r="H53" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ déroulé partagé avec le client</v>
       </c>
-      <c r="I53" s="22" t="str">
+      <c r="I53" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$61:$D$61,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="13" t="str">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="str">
         <f aca="false">Paramètres!A62</f>
         <v>PR-08 Restitution du lieu</v>
       </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="22" t="str">
+      <c r="B54" s="12"/>
+      <c r="C54" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="D54" s="22" t="str">
+      <c r="D54" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="E54" s="22" t="str">
+      <c r="E54" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="F54" s="22" t="str">
+      <c r="F54" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="G54" s="22" t="str">
+      <c r="G54" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="H54" s="22" t="str">
+      <c r="H54" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓</v>
       </c>
-      <c r="I54" s="22" t="str">
+      <c r="I54" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$62:$D$62,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="13" t="str">
+    <row r="55" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="14" t="str">
         <f aca="false">Paramètres!A63</f>
         <v>PR-09 Incident et plan B</v>
       </c>
-      <c r="B55" s="11"/>
-      <c r="C55" s="22" t="str">
+      <c r="B55" s="12"/>
+      <c r="C55" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓</v>
       </c>
-      <c r="D55" s="22" t="str">
+      <c r="D55" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓</v>
       </c>
-      <c r="E55" s="22" t="str">
+      <c r="E55" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓</v>
       </c>
-      <c r="F55" s="22" t="str">
+      <c r="F55" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓ + plan de communication de crise</v>
       </c>
-      <c r="G55" s="22" t="str">
+      <c r="G55" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓</v>
       </c>
-      <c r="H55" s="22" t="str">
+      <c r="H55" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓✓</v>
       </c>
-      <c r="I55" s="22" t="str">
+      <c r="I55" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$63:$D$63,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="13" t="str">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="str">
         <f aca="false">Paramètres!A64</f>
         <v>PR-10 Bilan</v>
       </c>
-      <c r="B56" s="11"/>
-      <c r="C56" s="22" t="str">
+      <c r="B56" s="12"/>
+      <c r="C56" s="23" t="str">
         <f aca="false">IF(C$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(C$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓ + retour du client</v>
       </c>
-      <c r="D56" s="22" t="str">
+      <c r="D56" s="23" t="str">
         <f aca="false">IF(D$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(D$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓ + retour du client</v>
       </c>
-      <c r="E56" s="22" t="str">
+      <c r="E56" s="23" t="str">
         <f aca="false">IF(E$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(E$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓ + retour du client</v>
       </c>
-      <c r="F56" s="22" t="str">
+      <c r="F56" s="23" t="str">
         <f aca="false">IF(F$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(F$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓ + revue de presse</v>
       </c>
-      <c r="G56" s="22" t="str">
+      <c r="G56" s="23" t="str">
         <f aca="false">IF(G$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(G$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓ + retour du client</v>
       </c>
-      <c r="H56" s="22" t="str">
+      <c r="H56" s="23" t="str">
         <f aca="false">IF(H$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(H$10,Paramètres!$B$54:$D$54,0)))</f>
         <v>✓ + retour du client</v>
       </c>
-      <c r="I56" s="22" t="str">
+      <c r="I56" s="23" t="str">
         <f aca="false">IF(I$10="","",INDEX(Paramètres!$B$64:$D$64,MATCH(I$10,Paramètres!$B$54:$D$54,0)))</f>
         <v/>
       </c>
@@ -2998,747 +2999,747 @@
   <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="24" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="25" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="25" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="25" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="25" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="25" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="24"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="D10" s="25"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="24"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
+      <c r="D12" s="25"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="25" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="24"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
+      <c r="D14" s="25"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="26" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="24" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="25" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="25" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="25" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="25" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B23" s="11" t="n">
         <v>100000</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="25" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="26" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="D27" s="23" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
+      <c r="B28" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B28" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="C28" s="11" t="s">
+      <c r="D28" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="D28" s="24" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" s="12" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
+      <c r="D29" s="25" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="26" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B34" s="27"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B35" s="27"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="25" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B36" s="27"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="25" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B37" s="27"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B38" s="27"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B39" s="27"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B40" s="27"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41" s="27"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="25" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42" s="27"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="25" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B43" s="27"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="25" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="B44" s="27"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="B45" s="27"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="25" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="B46" s="27"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="25" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B47" s="27"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="25" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B48" s="27"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="25" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="B49" s="27"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="26" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="B54" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D29" s="24" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12" t="s">
+      <c r="D54" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="D30" s="24" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="E33" s="23" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="B34" s="26"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="24" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="B35" s="26"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="24" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="B36" s="26"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="24" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="B37" s="26"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="24" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="B38" s="26"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="B39" s="26"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="24" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="B40" s="26"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="24" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="B41" s="26"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="24" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="B42" s="26"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="24" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="B43" s="26"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="24" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="B44" s="26"/>
-      <c r="C44" s="27"/>
-      <c r="D44" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" s="24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="B45" s="26"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" s="24" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B46" s="26"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="24" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="B47" s="26"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="24" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="B48" s="26"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="24" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="B49" s="26"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="24" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="23" t="s">
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="B54" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="C54" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="D54" s="23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="24" t="s">
+      <c r="B55" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="B55" s="24" t="s">
+      <c r="C55" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="C55" s="24" t="s">
+      <c r="D55" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="D55" s="24" t="s">
+    </row>
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="25" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="24" t="s">
+      <c r="B56" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="B56" s="24" t="s">
+      <c r="C56" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="C56" s="24" t="s">
+      <c r="D56" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="D56" s="24" t="s">
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="25" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="24" t="s">
+      <c r="B57" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C57" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="B57" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C57" s="24" t="s">
+      <c r="D57" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="D57" s="24" t="s">
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="24" t="s">
+      <c r="B58" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C58" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="B58" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C58" s="24" t="s">
+      <c r="D58" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="D58" s="24" t="s">
+    </row>
+    <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="25" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="24" t="s">
+      <c r="B59" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C59" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="B59" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C59" s="24" t="s">
+      <c r="D59" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="D59" s="24" t="s">
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="25" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="24" t="s">
+      <c r="B60" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C60" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D60" s="25" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="B60" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C60" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="D60" s="24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="24" t="s">
+      <c r="B61" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C61" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="B61" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C61" s="24" t="s">
+      <c r="D61" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="D61" s="24" t="s">
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="25" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="24" t="s">
+      <c r="B62" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C62" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D62" s="25" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="B62" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C62" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="D62" s="24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="24" t="s">
+      <c r="B63" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C63" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="B63" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C63" s="24" t="s">
+      <c r="D63" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="D63" s="24" t="s">
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="25" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="24" t="s">
+      <c r="B64" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="C64" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="B64" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="C64" s="24" t="s">
+      <c r="D64" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="D64" s="24" t="s">
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="26" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="25" t="s">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="29" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="28" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="29" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="28" t="s">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="29" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="28" t="s">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="29" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="28" t="s">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="28" t="s">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="29" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="28" t="s">
-        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Opérations : alignement sur les décisions D-02 à D-24 — enveloppe d'équipe de la Finance, vin selon le Juridique, wine maker dinner AdVini, Pop Tables, sans photographe, PMS prévu (29/10/2026)
- Staffing : l'enveloppe de la Finance (D-06) devient le budget de l'équipe ; effectif de référence, écarts, coût horaire permis, leviers et risques pour la qualité ; privatisation à 30 couverts (D-22)
- Vin : AdVini envoie un winemaker non rémunéré ; Pop Tables achète les vins et les vend sous sa licence (D-09, M04) ; sulfites, alcool, licence dans PR-01, PR-03 à PR-05 et PR-07
- Plan de maîtrise sanitaire prévu avant la pré-vente du premier pilote (PR-06, rétroplanning), non conçu
- « Fou d'un soir » remplacé par « Pop Tables » (D-03) ; photographe retiré (D-08)
- Note au Marketing et aux Ventes et notes de staffing renommées au 29/10/2026

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jw3cAUG7U3Lzwe6uXrNiNt
</commit_message>
<xml_diff>
--- a/6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx
+++ b/6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx
@@ -647,14 +647,14 @@
     <row r="1" ht="17.25" customHeight="1" s="31">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>Calculateur de staffing par événement — Fou d'un soir</t>
+          <t>Calculateur de staffing par événement — Pop Tables</t>
         </is>
       </c>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="31">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>28/10/2026 · 6 OPERATIONS/PRODUCTION · Document de travail du pôle Opérations : propositions, mis à jour le 28/10/2026 (jauges de la Finance, sans sommelier, équipe fixe) ; rien n'est décidé (voir REGISTRE DES DECISIONS).</t>
+          <t>28/10/2026, mis à jour le 29/10/2026 · 6 OPERATIONS/PRODUCTION · Document de travail du pôle Opérations : jauges de la Direction (D-05, D-22), pas de sommelier (wine maker dinner AdVini), pas de photographe (D-08). Le coût calculé est un effectif de référence ; le budget de l'équipe est l'enveloppe de la Finance (D-06).</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
     <row r="11" ht="23.25" customHeight="1" s="31">
       <c r="A11" s="34" t="inlineStr">
         <is>
-          <t>3. « Service de salle fourni par » : laisser « Nous ». Depuis le 28/10/2026, l'orientation du pôle Opérations est que Fou d'un soir fournit toujours le personnel (note de typologie, § 3.4). Le choix « Restaurant » n'est gardé que pour mémoire.</t>
+          <t>3. « Service de salle fourni par » : laisser « Nous ». Pop Tables fournit toujours le personnel (décision D-07 du 28/10/2026). Le choix « Restaurant » n'est gardé que pour mémoire.</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
     <row r="2" ht="15" customHeight="1" s="31">
       <c r="A2" s="37" t="inlineStr">
         <is>
-          <t>Ne saisir que les cellules jaunes (lignes 5 à 13). Exemples mis à jour le 28/10/2026 aux jauges du modèle de la Finance (40, 35, 30 et 20 couverts) : propositions, non décidées.</t>
+          <t>Ne saisir que les cellules jaunes (lignes 5 à 13). Exemples aux jauges de la Direction (D-05, D-22) : 40, 35 et 30 couverts à la place, 30 en privatisation.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="H5" s="41" t="inlineStr">
         <is>
-          <t>Privatisation (offre B)</t>
+          <t>Privatisation (30 couverts, D-22)</t>
         </is>
       </c>
       <c r="I5" s="41" t="inlineStr">
@@ -945,7 +945,7 @@
         <v>2</v>
       </c>
       <c r="H7" s="41" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I7" s="41" t="n">
         <v>40</v>
@@ -1937,31 +1937,31 @@
         <v/>
       </c>
       <c r="C37" s="43">
-        <f>IF(C$7="","",IF(C$10="C3",1,0))</f>
+        <f>IF(C$7="","",0)</f>
         <v/>
       </c>
       <c r="D37" s="43">
-        <f>IF(D$7="","",IF(D$10="C3",1,0))</f>
+        <f>IF(D$7="","",0)</f>
         <v/>
       </c>
       <c r="E37" s="43">
-        <f>IF(E$7="","",IF(E$10="C3",1,0))</f>
+        <f>IF(E$7="","",0)</f>
         <v/>
       </c>
       <c r="F37" s="43">
-        <f>IF(F$7="","",IF(F$10="C3",1,0))</f>
+        <f>IF(F$7="","",0)</f>
         <v/>
       </c>
       <c r="G37" s="43">
-        <f>IF(G$7="","",IF(G$10="C3",1,0))</f>
+        <f>IF(G$7="","",0)</f>
         <v/>
       </c>
       <c r="H37" s="43">
-        <f>IF(H$7="","",IF(H$10="C3",1,0))</f>
+        <f>IF(H$7="","",0)</f>
         <v/>
       </c>
       <c r="I37" s="43">
-        <f>IF(I$7="","",IF(I$10="C3",1,0))</f>
+        <f>IF(I$7="","",0)</f>
         <v/>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="D7" s="55" t="inlineStr">
         <is>
-          <t>En dessous, le sommelier tient la salle.</t>
+          <t>En dessous, le winemaker et le chef tiennent la salle (pas de sommelier depuis le 29/10/2026).</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="D9" s="55" t="inlineStr">
         <is>
-          <t>28/10/2026 : seuil porté de 20 à 21 couverts : la privatisation de 20 couverts n'a pas d'aide sommelier, comme en S3. Accords vins et jus servis en parallèle (offre du Produit).</t>
+          <t>Seuil de 21 couverts : pas d'aide sommelier en dessous. L'aide sommelier sert les accords vins et jus présentés par le winemaker d'AdVini.</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D15" s="55" t="inlineStr">
         <is>
-          <t>28/10/2026 : orientation du responsable Opérations : pas de sommelier. Le vigneron d'AdVini présente et vend lui-même son vin, sans être rémunéré (communication pour AdVini). Accord non signé à ce jour.</t>
+          <t>29/10/2026, orientation du responsable Opérations : pas de sommelier. AdVini envoie un winemaker (format « wine maker dinner ») qui conçoit et présente les accords, sans être rémunéré. Pop Tables achète les vins et les vend sous sa propre licence (D-09 ; contrat M04 du Juridique). Accord avec AdVini non signé à ce jour.</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="E40" s="55" t="inlineStr">
         <is>
-          <t>1 par événement si le paramètre « Sommelier invité payé par nous » vaut 1 (0 depuis le 28/10/2026 : vigneron d'AdVini).</t>
+          <t>1 par événement si le paramètre « Sommelier invité payé par nous » vaut 1 (0 depuis le 29/10/2026 : winemaker d'AdVini, non rémunéré).</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
     <row r="47" ht="15" customHeight="1" s="31">
       <c r="A47" s="42" t="inlineStr">
         <is>
-          <t>Photographe</t>
+          <t>Photographe (supprimé, D-08)</t>
         </is>
       </c>
       <c r="B47" s="57" t="n"/>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E47" s="55" t="inlineStr">
         <is>
-          <t>1 en C3 (prévu dans les trois options de lancement du Marketing).</t>
+          <t>0 : pas de photographe par soirée (décision D-08 du 28/10/2026).</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
     <row r="50" ht="15" customHeight="1" s="31">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>H : heures et coûts horaires repris du modèle Prévisions de la Finance (onglet « Staffing », 28/10/2026), à remplacer par les devis d'une agence d'extras. Rôles C3 (accueil, presse, photographe, vidéaste, logistique) non chiffrés : le coût de la colonne Lancement est donc sous-estimé.</t>
+          <t>H : heures et coûts horaires repris du modèle de la Finance (onglet « Staffing »), à remplacer par les devis. Le coût calculé sert de référence : le budget de l'équipe est l'enveloppe de la Finance (D-06), 15 ou 20 % du CA HT. Rôles C3 (accueil, presse, vidéaste, logistique) non chiffrés.</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
     <row r="72" ht="15" customHeight="1" s="31">
       <c r="A72" s="59" t="inlineStr">
         <is>
-          <t>Formats d'événements : 5 PRODUIT/Fou d'un soir l'offre.md et plan des deux soirées pilotes (27/10/2026) ; 3 MARKETING/new project/9 Premier événement/2026 1028 Premier événement - Trois options.md</t>
+          <t>Formats d'événements : 5 PRODUIT/2026 1028 Pop Tables - Offre.md et Pop Tables - Pricing.md (28/10/2026) ; décisions D-05 et D-22 (jauges) ; 3 MARKETING/new project/9 Premier événement/2026 1028 Premier événement - Trois options.md</t>
         </is>
       </c>
     </row>

</xml_diff>